<commit_message>
SE calculations for Query ACS data script, added BLS post-processing work, included Accessibility_4 and Accessibility_2 and Income_2 post-processing scripts
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\Census\aa_config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE3F1215-FC89-4FF7-9075-FFC0466AC534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08092D6D-55C1-4E3E-81D4-A2BA58E12352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicators" sheetId="5" r:id="rId1"/>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="185">
   <si>
     <t>Indicator</t>
   </si>
@@ -715,12 +715,30 @@
   <si>
     <t>Metric is tracked on the household, not individual, level</t>
   </si>
+  <si>
+    <t>Accessibility_2</t>
+  </si>
+  <si>
+    <t>Travel Mode by Household Income</t>
+  </si>
+  <si>
+    <t>Accessibility_4</t>
+  </si>
+  <si>
+    <t>Commute Time</t>
+  </si>
+  <si>
+    <t>Accessibility_1</t>
+  </si>
+  <si>
+    <t>Travel Mode by Race</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -780,12 +798,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1221,11 +1233,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E88C108-3781-4F95-A6AF-A4204BCDFF66}">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -1602,6 +1614,30 @@
       </c>
       <c r="B47" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>183</v>
+      </c>
+      <c r="B48" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>181</v>
+      </c>
+      <c r="B50" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -3048,6 +3084,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -3276,15 +3321,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3297,6 +3333,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CDC4E648-E9B1-485C-B58B-225AE7E05985}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3315,14 +3359,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Condensed Query ACS Data script into separate functions, finalized exporting to csv script
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08092D6D-55C1-4E3E-81D4-A2BA58E12352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F6EF51-A5D4-48E2-B6B1-F4A59D285391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="189">
   <si>
     <t>Indicator</t>
   </si>
@@ -732,6 +732,18 @@
   </si>
   <si>
     <t>Travel Mode by Race</t>
+  </si>
+  <si>
+    <t>Health_1</t>
+  </si>
+  <si>
+    <t>Access to Grocery Stores</t>
+  </si>
+  <si>
+    <t>Accessibility_3</t>
+  </si>
+  <si>
+    <t>Auto Ownership</t>
   </si>
 </sst>
 </file>
@@ -1233,7 +1245,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E88C108-3781-4F95-A6AF-A4204BCDFF66}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
@@ -1290,353 +1302,369 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>185</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>139</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>183</v>
+        <v>139</v>
       </c>
       <c r="B48" t="s">
-        <v>184</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B50" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>187</v>
+      </c>
+      <c r="B51" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>181</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B52" t="s">
         <v>182</v>
       </c>
     </row>
@@ -3084,12 +3112,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3322,20 +3352,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
+    <ds:schemaRef ds:uri="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3360,12 +3391,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
-    <ds:schemaRef ds:uri="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Major changes to organization of census preparation scripts, fixed PUMS query pulls for persons and households merging files, started FOODSEC query
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F6EF51-A5D4-48E2-B6B1-F4A59D285391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFAD9B25-99F7-4B14-8459-F0A13820A854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="192">
   <si>
     <t>Indicator</t>
   </si>
@@ -744,6 +744,15 @@
   </si>
   <si>
     <t>Auto Ownership</t>
+  </si>
+  <si>
+    <t>MOE Threshold</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Not sure if I can pull SE's yet</t>
   </si>
 </sst>
 </file>
@@ -1245,427 +1254,584 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E88C108-3781-4F95-A6AF-A4204BCDFF66}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C1" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>185</v>
       </c>
       <c r="B7" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>24</v>
       </c>
       <c r="B14" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
       <c r="B15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C15" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>30</v>
       </c>
       <c r="B17" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>34</v>
       </c>
       <c r="B19" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>36</v>
       </c>
       <c r="B20" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C20" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>38</v>
       </c>
       <c r="B21" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>40</v>
       </c>
       <c r="B22" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>42</v>
       </c>
       <c r="B23" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C23" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>44</v>
       </c>
       <c r="B24" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C24" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>46</v>
       </c>
       <c r="B25" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C25" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>48</v>
       </c>
       <c r="B26" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>50</v>
       </c>
       <c r="B27" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>52</v>
       </c>
       <c r="B28" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>54</v>
       </c>
       <c r="B29" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>56</v>
       </c>
       <c r="B30" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>58</v>
       </c>
       <c r="B31" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>59</v>
       </c>
       <c r="B32" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>61</v>
       </c>
       <c r="B33" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>63</v>
       </c>
       <c r="B34" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C34" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>65</v>
       </c>
       <c r="B35" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C35" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>67</v>
       </c>
       <c r="B36" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C36" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>69</v>
       </c>
       <c r="B37" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C37" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>71</v>
       </c>
       <c r="B38" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>73</v>
       </c>
       <c r="B39" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>75</v>
       </c>
       <c r="B40" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>77</v>
       </c>
       <c r="B41" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>79</v>
       </c>
       <c r="B42" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C42" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>81</v>
       </c>
       <c r="B43" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>83</v>
       </c>
       <c r="B44" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C44">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>85</v>
       </c>
       <c r="B45" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>87</v>
       </c>
       <c r="B46" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C46" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>89</v>
       </c>
       <c r="B47" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C47" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>139</v>
       </c>
       <c r="B48" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C48">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>183</v>
       </c>
       <c r="B49" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>179</v>
       </c>
       <c r="B50" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C50">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>187</v>
       </c>
       <c r="B51" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C51">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>181</v>
       </c>
       <c r="B52" t="s">
         <v>182</v>
+      </c>
+      <c r="C52">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3112,14 +3278,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3352,21 +3516,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
-    <ds:schemaRef ds:uri="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3391,9 +3554,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
+    <ds:schemaRef ds:uri="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Major updates to PUMS processing
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFAD9B25-99F7-4B14-8459-F0A13820A854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CCFF36-CA78-43DF-83B8-F5CB99F414B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -725,9 +725,6 @@
     <t>Accessibility_4</t>
   </si>
   <si>
-    <t>Commute Time</t>
-  </si>
-  <si>
     <t>Accessibility_1</t>
   </si>
   <si>
@@ -753,6 +750,9 @@
   </si>
   <si>
     <t>Not sure if I can pull SE's yet</t>
+  </si>
+  <si>
+    <t>Commute Times</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1270,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1281,7 +1281,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1292,7 +1292,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1325,18 +1325,18 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" t="s">
         <v>185</v>
       </c>
-      <c r="B7" t="s">
-        <v>186</v>
-      </c>
       <c r="C7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1391,7 +1391,7 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -1402,7 +1402,7 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -1424,7 +1424,7 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -1457,7 +1457,7 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -1468,7 +1468,7 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -1479,7 +1479,7 @@
         <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -1490,7 +1490,7 @@
         <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -1501,7 +1501,7 @@
         <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -1512,7 +1512,7 @@
         <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -1523,7 +1523,7 @@
         <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -1534,7 +1534,7 @@
         <v>47</v>
       </c>
       <c r="C25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -1545,7 +1545,7 @@
         <v>49</v>
       </c>
       <c r="C26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -1556,7 +1556,7 @@
         <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -1567,7 +1567,7 @@
         <v>53</v>
       </c>
       <c r="C28" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -1578,7 +1578,7 @@
         <v>55</v>
       </c>
       <c r="C29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -1589,7 +1589,7 @@
         <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -1600,7 +1600,7 @@
         <v>51</v>
       </c>
       <c r="C31" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -1611,7 +1611,7 @@
         <v>60</v>
       </c>
       <c r="C32" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
@@ -1622,7 +1622,7 @@
         <v>62</v>
       </c>
       <c r="C33" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -1633,7 +1633,7 @@
         <v>64</v>
       </c>
       <c r="C34" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -1644,7 +1644,7 @@
         <v>66</v>
       </c>
       <c r="C35" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -1655,7 +1655,7 @@
         <v>68</v>
       </c>
       <c r="C36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1666,7 +1666,7 @@
         <v>70</v>
       </c>
       <c r="C37" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -1721,7 +1721,7 @@
         <v>80</v>
       </c>
       <c r="C42" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1765,7 +1765,7 @@
         <v>88</v>
       </c>
       <c r="C46" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1776,7 +1776,7 @@
         <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -1792,10 +1792,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>182</v>
+      </c>
+      <c r="B49" t="s">
         <v>183</v>
-      </c>
-      <c r="B49" t="s">
-        <v>184</v>
       </c>
       <c r="C49">
         <v>5</v>
@@ -1814,10 +1814,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>186</v>
+      </c>
+      <c r="B51" t="s">
         <v>187</v>
-      </c>
-      <c r="B51" t="s">
-        <v>188</v>
       </c>
       <c r="C51">
         <v>5</v>
@@ -1828,7 +1828,7 @@
         <v>181</v>
       </c>
       <c r="B52" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C52">
         <v>5</v>
@@ -3278,15 +3278,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -3515,6 +3506,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3527,14 +3527,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CDC4E648-E9B1-485C-B58B-225AE7E05985}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3553,6 +3545,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Major updates to CPS script, started Housing Production indicators
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CCFF36-CA78-43DF-83B8-F5CB99F414B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8DD70D1-9A7E-4646-B271-B97F6574704A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicators" sheetId="5" r:id="rId1"/>
@@ -20,14 +20,23 @@
     <sheet name="Pop_4" sheetId="7" r:id="rId5"/>
     <sheet name="Pop_5" sheetId="3" r:id="rId6"/>
     <sheet name="Labor_1" sheetId="4" r:id="rId7"/>
-    <sheet name="Cost_5" sheetId="8" r:id="rId8"/>
-    <sheet name="Cost_6" sheetId="9" r:id="rId9"/>
-    <sheet name="Income_1" sheetId="10" r:id="rId10"/>
-    <sheet name="Income_2" sheetId="11" r:id="rId11"/>
-    <sheet name="Income_3" sheetId="12" r:id="rId12"/>
-    <sheet name="Edu_1" sheetId="13" r:id="rId13"/>
-    <sheet name="Health_2" sheetId="14" r:id="rId14"/>
-    <sheet name="Broadband_2" sheetId="15" r:id="rId15"/>
+    <sheet name="Labor_2" sheetId="18" r:id="rId8"/>
+    <sheet name="Cost_3" sheetId="20" r:id="rId9"/>
+    <sheet name="Cost_5" sheetId="8" r:id="rId10"/>
+    <sheet name="Cost_6" sheetId="9" r:id="rId11"/>
+    <sheet name="Income_1" sheetId="17" r:id="rId12"/>
+    <sheet name="Income_2" sheetId="11" r:id="rId13"/>
+    <sheet name="Income_3" sheetId="12" r:id="rId14"/>
+    <sheet name="Income_4" sheetId="19" r:id="rId15"/>
+    <sheet name="Edu_1" sheetId="13" r:id="rId16"/>
+    <sheet name="Health_1" sheetId="16" r:id="rId17"/>
+    <sheet name="Health_2" sheetId="14" r:id="rId18"/>
+    <sheet name="Broadband_2" sheetId="15" r:id="rId19"/>
+    <sheet name="Accessibility_1" sheetId="21" r:id="rId20"/>
+    <sheet name="Accessibility_2" sheetId="22" r:id="rId21"/>
+    <sheet name="Accessibility_3" sheetId="23" r:id="rId22"/>
+    <sheet name="Accessibility_4" sheetId="24" r:id="rId23"/>
+    <sheet name="Commute_1" sheetId="26" r:id="rId24"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -49,47 +58,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={B2DC7857-FFA8-44CC-BF4D-C43F18B06D21}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{B2DC7857-FFA8-44CC-BF4D-C43F18B06D21}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    @Joshua Fontes for this Income_2, doesnt look like the outputs through time have been adjusted for inflation. Is that the case? If so, we would want to adjust in inflation-adjusted dollars</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={1F1D5D9E-ABED-426C-80F8-5B6D62A91504}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-[Tasks]
-There is a task anchored to this comment that cannot be viewed in your client.
-Comment:
-    @Joshua Fontes can we also pull this Health_2 at the 1 year ACS.
-Per our decision tree, dont need anything below region level for 1 year ACS (ie dont need tracts and counties, just MPO)</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="238">
   <si>
     <t>Indicator</t>
   </si>
@@ -527,18 +497,9 @@
     <t>Labor Force</t>
   </si>
   <si>
-    <t>Census Bureau American Community Survey</t>
-  </si>
-  <si>
     <t>2009-2022</t>
   </si>
   <si>
-    <t>Estimated population in the labor force by race/ethnicity</t>
-  </si>
-  <si>
-    <t>Tracts and Counties</t>
-  </si>
-  <si>
     <t>American Community Survey (ACS) (census.gov)</t>
   </si>
   <si>
@@ -617,9 +578,6 @@
     <t>The indicator is measured at the household (not individual) level.</t>
   </si>
   <si>
-    <t>Margin of Error</t>
-  </si>
-  <si>
     <t>Housing Cost Burden by Race/Ethnicity</t>
   </si>
   <si>
@@ -668,21 +626,12 @@
     <t>5 year rolling average of % of households within income categories</t>
   </si>
   <si>
-    <t>SACOG region (MPO), and counties and tracts within</t>
-  </si>
-  <si>
     <t>Median Household Income by Race/Ethnicity</t>
   </si>
   <si>
     <t>5 year rolling average of median housheold income by Census Bureau race and ethnicity categories</t>
   </si>
   <si>
-    <t>SACOG (region) and counties</t>
-  </si>
-  <si>
-    <t>The indicator is nominal (not inflation-adjusted) dollars</t>
-  </si>
-  <si>
     <t>The indicator compares the median household income by individual race/ethnicities to the regional average. A value above 1 means the groups has a median household income above regional median (while below 1 means below regional level)</t>
   </si>
   <si>
@@ -734,9 +683,6 @@
     <t>Health_1</t>
   </si>
   <si>
-    <t>Access to Grocery Stores</t>
-  </si>
-  <si>
     <t>Accessibility_3</t>
   </si>
   <si>
@@ -749,17 +695,179 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Not sure if I can pull SE's yet</t>
-  </si>
-  <si>
     <t>Commute Times</t>
+  </si>
+  <si>
+    <t>Food Security</t>
+  </si>
+  <si>
+    <t>Access to grocery stores by Race/Ethnicity</t>
+  </si>
+  <si>
+    <t>Census 1 Year CPS (American Community Survey)</t>
+  </si>
+  <si>
+    <t>SACOG counties</t>
+  </si>
+  <si>
+    <t>CPS Supplement and Replicate Weights (census.gov)</t>
+  </si>
+  <si>
+    <t>HES1A:</t>
+  </si>
+  <si>
+    <t>Expend shopped at supermarket/grocery store last week</t>
+  </si>
+  <si>
+    <t>HES1B:</t>
+  </si>
+  <si>
+    <t>Expend shopped at dollar stores, pharmacies, etc.</t>
+  </si>
+  <si>
+    <t>Unemployment Rate</t>
+  </si>
+  <si>
+    <t>Bureau of Labor Statistics</t>
+  </si>
+  <si>
+    <t>Census 5 year ACS PUMS (Public Use Microdata Sample)</t>
+  </si>
+  <si>
+    <t>2016-2022</t>
+  </si>
+  <si>
+    <t>American Community Survey Microdata (census.gov)</t>
+  </si>
+  <si>
+    <t>The indicator measures household income in 2023 inflation adjusted dollars ($)</t>
+  </si>
+  <si>
+    <t>CPI Inflation Adjustment Factors.xlsx (sharepoint.com)</t>
+  </si>
+  <si>
+    <t>The income brackets (Low, Moderate, and High) are organized uniquely to each county, using the state guidelines</t>
+  </si>
+  <si>
+    <t>Income Limits 2023 (ca.gov)</t>
+  </si>
+  <si>
+    <t>SACOG region (MPO)</t>
+  </si>
+  <si>
+    <t>The indicator is in inflation-adjusted dollars</t>
+  </si>
+  <si>
+    <t>Poverty rate by race/ethnicity</t>
+  </si>
+  <si>
+    <t>5 year rolling average of % of households within census federal definition of poverty</t>
+  </si>
+  <si>
+    <t>Measures households living in poverty using the census official poverty measure. The census poverty measure compares pretax money to a threshold adjusted by family size and for inflation through time. Importantly, the Census Bureau uses the same poverty threshold throughout the United States, which does not fully reflect the effect of high housing costs in states such as California. Recognizing this limitation, the monitoring program uses the indicator for a relative comparison across race/ethnicity.</t>
+  </si>
+  <si>
+    <t>5 year rolling average of working age population in the formal labor force, by race/ethnicity</t>
+  </si>
+  <si>
+    <t>SACOG Region (MPO)</t>
+  </si>
+  <si>
+    <t>Unoccupied Housing Units</t>
+  </si>
+  <si>
+    <t>5 year rolling average of residential housing occupancy</t>
+  </si>
+  <si>
+    <t>The indicator estimates occupancy of the residential housing stock using three categories: occupied, vacant (for rent, for sale, otherwise not occupied, and occasional/seasonal use (vacation homes, etc).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margin of Error: all ACS outputs are estimates. The downloadable data includes the margin of error statistics. Users should pay particular attention to the margin of error, especially for smaller geographies and race/ethnicity groups with relatively less population. </t>
+  </si>
+  <si>
+    <t>There are four possible pairings from these categories</t>
+  </si>
+  <si>
+    <t>HES1b</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Used both supermarkets and dollar stores/pharmacies/convenience stores within last week for food purchases</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Exclusively used supermarket/grocery store in last week for food purchases</t>
+  </si>
+  <si>
+    <t>Exclusively used dollar store/pharmacy/convenience store last week for food purchase</t>
+  </si>
+  <si>
+    <t>Did not make food purchase last week</t>
+  </si>
+  <si>
+    <t>Counties</t>
+  </si>
+  <si>
+    <t>Estimated unemployment rate by counties</t>
+  </si>
+  <si>
+    <t>2000-2022</t>
+  </si>
+  <si>
+    <t>Commute modes by race/ethnicity</t>
+  </si>
+  <si>
+    <t>Census PUMS, 5 year ACS</t>
+  </si>
+  <si>
+    <t>Commute modes by income bracket</t>
+  </si>
+  <si>
+    <t>5 year rolling average of head of household commute modes by income bracket</t>
+  </si>
+  <si>
+    <t>2016-2021</t>
+  </si>
+  <si>
+    <t>Vehicle ownership by household</t>
+  </si>
+  <si>
+    <t>The indicator is measured at the household level</t>
+  </si>
+  <si>
+    <t>Yearly estimate of head of commute modes by race/ethnicity</t>
+  </si>
+  <si>
+    <t>The indicator is measured at the person level</t>
+  </si>
+  <si>
+    <t>5 year rolling average of household vehicle ownership</t>
+  </si>
+  <si>
+    <t>Commute times by income bracket and by race/ethnicity</t>
+  </si>
+  <si>
+    <t>5 year rolling average of head of household commute times by income bracket and by race/ethnicity</t>
+  </si>
+  <si>
+    <t>Estimate Mode of Commute through time</t>
+  </si>
+  <si>
+    <t>5 year rolling average of estimated travel mode to work</t>
+  </si>
+  <si>
+    <t>2009-2022 estimate at the SACOG region MPO level by race/ethnicity categories</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -821,6 +929,19 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -830,12 +951,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -844,7 +980,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -855,6 +991,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -872,46 +1011,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
-  <Task id="{7A5BE5EA-0CA6-410A-87BD-31E93D3E4870}">
-    <Anchor>
-      <Comment id="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}"/>
-    </Anchor>
-    <History>
-      <Event time="2024-06-05T22:36:26.40" id="{7E826F37-E978-4BEF-8283-0CF6F25CCD41}">
-        <Attribution userId="" userName="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Policies\Microsoft\Win" userProvider="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Microsoft\Windows\Curr"/>
-        <Anchor>
-          <Comment id="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}"/>
-        </Anchor>
-        <Create/>
-      </Event>
-      <Event time="2024-06-05T22:36:26.40" id="{576F53AB-6E29-412C-82DA-2743A28E8DE8}">
-        <Attribution userId="" userName="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Policies\Microsoft\Win" userProvider="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Microsoft\Windows\Curr"/>
-        <Anchor>
-          <Comment id="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}"/>
-        </Anchor>
-        <Assign userId="REGISTRY\MACHINE\Software\Microsoft\Windows\CurrentVersion\Explorer\Desktop\NameSpace\{031E4" userName="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Microsoft\Windows\Curr" userProvider="REGISTRY\MACHINE\Software\Microsoft\Windows\CurrentVersion\Explorer\Desktop\NameSpace\{F02C1"/>
-      </Event>
-      <Event time="2024-06-05T22:36:26.40" id="{AC979172-2D6A-4FB2-AFCD-B3F22A51DA63}">
-        <Attribution userId="" userName="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Policies\Microsoft\Win" userProvider="REGISTRY\USER\S-1-5-21-1935655697-790525478-1801674531-14204\Software\Microsoft\Windows\Curr"/>
-        <Anchor>
-          <Comment id="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}"/>
-        </Anchor>
-        <SetTitle title="@Joshua Fontes can we also pull this Health_2 at the 1 year ACS. Per our decision tree, dont need anything below region level for 1 year ACS (ie dont need tracts and counties, just MPO)"/>
-      </Event>
-    </History>
-  </Task>
-</Tasks>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Joshua Fontes" id="{8B5350AE-6FBA-4684-99B7-407DBD0ADFE4}" userId="jfontes@sacog.org" providerId="PeoplePicker"/>
-  <person displayName="Garett Ballard-Rosa" id="{99F2B82C-3921-49B1-91BB-A1BEBAE08438}" userId="S::gballard@sacog.org::a3ced981-b971-479c-b3fc-ef3dcb451512" providerId="AD"/>
-</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1229,29 +1328,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2024-06-11T22:34:24.95" personId="{99F2B82C-3921-49B1-91BB-A1BEBAE08438}" id="{B2DC7857-FFA8-44CC-BF4D-C43F18B06D21}">
-    <text>@Joshua Fontes for this Income_2, doesnt look like the outputs through time have been adjusted for inflation. Is that the case? If so, we would want to adjust in inflation-adjusted dollars</text>
-    <mentions>
-      <mention mentionpersonId="{8B5350AE-6FBA-4684-99B7-407DBD0ADFE4}" mentionId="{C7A7DC84-DA9B-42A6-88F8-DF985C554D77}" startIndex="0" length="14"/>
-    </mentions>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2024-06-05T22:36:26.44" personId="{99F2B82C-3921-49B1-91BB-A1BEBAE08438}" id="{1F1D5D9E-ABED-426C-80F8-5B6D62A91504}">
-    <text>@Joshua Fontes can we also pull this Health_2 at the 1 year ACS.
-Per our decision tree, dont need anything below region level for 1 year ACS (ie dont need tracts and counties, just MPO)</text>
-    <mentions>
-      <mention mentionpersonId="{8B5350AE-6FBA-4684-99B7-407DBD0ADFE4}" mentionId="{8AE4D7E0-E435-47C0-8FCF-F7071B7B2E6E}" startIndex="0" length="14"/>
-    </mentions>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E88C108-3781-4F95-A6AF-A4204BCDFF66}">
   <dimension ref="A1:C52"/>
@@ -1270,7 +1346,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1281,7 +1357,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1292,7 +1368,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1325,18 +1401,18 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1391,7 +1467,7 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -1402,7 +1478,7 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -1424,7 +1500,7 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -1457,7 +1533,7 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -1468,7 +1544,7 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -1479,7 +1555,7 @@
         <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -1490,7 +1566,7 @@
         <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -1501,7 +1577,7 @@
         <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -1512,7 +1588,7 @@
         <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -1523,7 +1599,7 @@
         <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -1534,7 +1610,7 @@
         <v>47</v>
       </c>
       <c r="C25" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -1545,7 +1621,7 @@
         <v>49</v>
       </c>
       <c r="C26" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -1556,7 +1632,7 @@
         <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -1567,7 +1643,7 @@
         <v>53</v>
       </c>
       <c r="C28" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -1578,7 +1654,7 @@
         <v>55</v>
       </c>
       <c r="C29" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -1589,7 +1665,7 @@
         <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -1600,7 +1676,7 @@
         <v>51</v>
       </c>
       <c r="C31" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -1611,7 +1687,7 @@
         <v>60</v>
       </c>
       <c r="C32" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
@@ -1622,7 +1698,7 @@
         <v>62</v>
       </c>
       <c r="C33" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -1633,7 +1709,7 @@
         <v>64</v>
       </c>
       <c r="C34" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -1644,7 +1720,7 @@
         <v>66</v>
       </c>
       <c r="C35" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -1655,7 +1731,7 @@
         <v>68</v>
       </c>
       <c r="C36" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1666,7 +1742,7 @@
         <v>70</v>
       </c>
       <c r="C37" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -1721,7 +1797,7 @@
         <v>80</v>
       </c>
       <c r="C42" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1765,7 +1841,7 @@
         <v>88</v>
       </c>
       <c r="C46" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1776,15 +1852,15 @@
         <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C48">
         <v>5</v>
@@ -1792,10 +1868,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="B49" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="C49">
         <v>5</v>
@@ -1803,10 +1879,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="B50" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C50">
         <v>5</v>
@@ -1814,10 +1890,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B51" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C51">
         <v>5</v>
@@ -1825,10 +1901,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="B52" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="C52">
         <v>5</v>
@@ -1840,114 +1916,121 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4BC3ADC-B173-4F45-B836-D1F7E22CED4E}">
-  <dimension ref="A1:B15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013C4FE6-69F4-4786-9394-986C84D07B5F}">
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+        <v>125</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B7" s="4">
-        <v>45413</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>45457</v>
+      </c>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>160</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{DE4D29F9-07A9-4120-8B12-72E55D9E43F5}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{58C581DA-D03C-4E16-9B4D-211D2C0C873B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FC9227-AA24-4EC1-82B7-529B992D0DA5}">
-  <dimension ref="A1:B13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71A9E054-EC73-4216-9E03-BD67B6393576}">
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
@@ -1958,7 +2041,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -1966,7 +2049,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1974,7 +2057,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1982,7 +2065,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -1990,7 +2073,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -1998,7 +2081,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2010,43 +2093,150 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{A51F4BBE-DD68-4C28-A93E-CE1114969021}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{54F56070-B8CC-4D8B-AFD0-D98EB20575C3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE77370-5B89-4A67-8993-8895C81279C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1E54E8F-CCF0-44C5-9CA6-76927E8C20C4}">
   <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45460</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{F5DAAD68-13E7-40D5-B343-5F9E4C88D373}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FC9227-AA24-4EC1-82B7-529B992D0DA5}">
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
@@ -2057,7 +2247,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2065,7 +2255,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2073,7 +2263,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2081,7 +2271,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2089,7 +2279,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2097,7 +2287,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2105,49 +2295,283 @@
         <v>103</v>
       </c>
       <c r="B7" s="4">
-        <v>45413</v>
+        <v>45495</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>168</v>
+      <c r="B10" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>132</v>
+      <c r="B12" s="3" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>133</v>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{5E0916F8-4257-4F52-B926-2A422DA3AD65}"/>
+    <hyperlink ref="B6" r:id="rId1" display="https://www.census.gov/programs-surveys/acs/microdata.html" xr:uid="{9F285AB3-D189-4735-8A27-F9D668EEB07F}"/>
+    <hyperlink ref="B10" r:id="rId2" display="../../../../../../../../:x:/r/sites/RegionalMonitoringandReporting/_layouts/15/Doc.aspx?sourcedoc=%7B88580A50-9A81-4CE5-A645-1260CD41BBF2%7D&amp;file=CPI%20Inflation%20Adjustment%20Factors.xlsx&amp;action=default&amp;mobileredirect=true&amp;wdsle=0" xr:uid="{3E357F10-3CB6-4A25-8AAC-BCFD6772D3E4}"/>
+    <hyperlink ref="B12" r:id="rId3" display="https://www.hcd.ca.gov/sites/default/files/docs/grants-and-funding/income-limits-2023.pdf" xr:uid="{A2CBD52A-3744-46D2-804A-C3C63BA54073}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE77370-5B89-4A67-8993-8895C81279C7}">
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45495</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{7F483C3D-2FDC-4854-8A26-A165FAE97C63}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7CDBA1-36C5-44A0-8A93-C60C2735B32B}">
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45461</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{08BE1AEB-40FC-40FC-B0D0-4CE6FDD4BA1C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410719E2-626B-4B5A-841A-284292C3B297}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2160,7 +2584,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2168,7 +2592,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2176,7 +2600,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2184,7 +2608,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2192,7 +2616,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2200,7 +2624,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2212,39 +2636,44 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2255,8 +2684,166 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65DE0E5F-735A-4F56-AE85-1C77154B186E}">
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B23FC43A-2DE6-4C9F-97EC-3AE395296ECB}">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45495</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C10" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B13" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B14" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B15" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B16" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>219</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" display="https://www.census.gov/data/datasets/time-series/demo/cps/cps-supp_cps-repwgt.html" xr:uid="{9DF484F8-4321-4052-A5B5-6D3CA9E2DFB7}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65DE0E5F-735A-4F56-AE85-1C77154B186E}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2268,7 +2855,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2276,7 +2863,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2284,7 +2871,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2292,7 +2879,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2300,7 +2887,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2308,7 +2895,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2320,7 +2907,12 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
@@ -2329,17 +2921,17 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2347,11 +2939,10 @@
     <hyperlink ref="B6" r:id="rId1" xr:uid="{D7B7E773-7A91-495D-9518-0977756B2F20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB03DB03-8A0F-452D-AAB6-A6D974594CE6}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2364,7 +2955,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2372,7 +2963,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2380,7 +2971,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2388,7 +2979,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2396,7 +2987,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2404,7 +2995,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2416,39 +3007,44 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2552,12 +3148,560 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2629891-FE09-42D3-A38D-F6AF2F47CE1F}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{8EC6BB2B-78ED-48AD-BB67-D30BEE0DC85D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2311C843-1F7B-44AA-8B7A-83C5EE5E8943}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{03028305-D390-4DE3-85E9-2940EF3E85AD}"/>
+    <hyperlink ref="B10" r:id="rId2" display="../../../../../../../../:x:/r/sites/RegionalMonitoringandReporting/_layouts/15/Doc.aspx?sourcedoc=%7B88580A50-9A81-4CE5-A645-1260CD41BBF2%7D&amp;file=CPI%20Inflation%20Adjustment%20Factors.xlsx&amp;action=default&amp;mobileredirect=true&amp;wdsle=0" xr:uid="{34C0CC81-4D1C-4F52-9167-4CCF735D426A}"/>
+    <hyperlink ref="B12" r:id="rId3" display="https://www.hcd.ca.gov/sites/default/files/docs/grants-and-funding/income-limits-2023.pdf" xr:uid="{9002450C-B6CE-419F-B189-4B5EC467912E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988B1DED-B96D-4459-B33A-3A22EEA612DF}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{DA8371B2-2EF5-40F6-9DD8-53A811D3E4BB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF115ED2-4ECF-4CB0-981E-7FC2A0734299}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45496</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{1BB89EB1-3974-4AEB-B1DD-AE7B10F2DE82}"/>
+    <hyperlink ref="B10" r:id="rId2" display="../../../../../../../../:x:/r/sites/RegionalMonitoringandReporting/_layouts/15/Doc.aspx?sourcedoc=%7B88580A50-9A81-4CE5-A645-1260CD41BBF2%7D&amp;file=CPI%20Inflation%20Adjustment%20Factors.xlsx&amp;action=default&amp;mobileredirect=true&amp;wdsle=0" xr:uid="{BC10A01F-E8D9-4D24-8580-C8D8068DEB81}"/>
+    <hyperlink ref="B12" r:id="rId3" display="https://www.hcd.ca.gov/sites/default/files/docs/grants-and-funding/income-limits-2023.pdf" xr:uid="{336E47FB-78AB-40BA-B603-89DEF6DFB1F6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06F0CF63-2338-427D-9D91-2A36269AF285}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45457</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{038D776C-3E83-417E-AB3F-397E3004703A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4D6AA6A-B6EF-493C-80CB-2138C013DFDD}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2657,13 +3801,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCD1F30-8321-44A7-AC64-59DE7A71B2E6}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2671,7 +3818,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2679,7 +3826,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2687,7 +3834,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2695,7 +3842,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2703,7 +3850,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2715,39 +3862,44 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2763,7 +3915,7 @@
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2771,7 +3923,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2779,7 +3931,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2787,7 +3939,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2795,7 +3947,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2803,7 +3955,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2811,7 +3963,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2823,39 +3975,44 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2971,6 +4128,123 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8B131F-D980-496F-9D95-BB5930E5D617}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45460</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" s="6"/>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" display="https://www.census.gov/programs-surveys/acs" xr:uid="{57066AFA-A39F-4D50-9FCF-D401C43CDB7E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD84412C-D52C-4EC3-8513-94B68EEC5106}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2983,7 +4257,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2991,7 +4265,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2999,7 +4273,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -3007,7 +4281,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -3015,16 +4289,14 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>120</v>
-      </c>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3035,43 +4307,27 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B9" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>123</v>
-      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" s="6"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" display="https://www.census.gov/programs-surveys/acs" xr:uid="{E30D7D86-05D6-465A-AE47-50DEAE2A3969}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013C4FE6-69F4-4786-9394-986C84D07B5F}">
-  <dimension ref="A1:F15"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0189621C-4234-46C7-973A-777F36522DAB}">
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -3079,7 +4335,7 @@
         <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>141</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -3087,7 +4343,7 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -3095,7 +4351,7 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -3103,7 +4359,7 @@
         <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -3111,7 +4367,7 @@
         <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -3119,7 +4375,7 @@
         <v>101</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F6" s="7"/>
     </row>
@@ -3128,150 +4384,42 @@
         <v>103</v>
       </c>
       <c r="B7" s="4">
-        <v>45413</v>
+        <v>45461</v>
       </c>
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
+      <c r="A8" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>145</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
+      <c r="F12" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{D455A751-D8D7-4066-BFFF-1AAFE34770F9}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71A9E054-EC73-4216-9E03-BD67B6393576}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="4">
-        <v>45413</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>155</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{54F56070-B8CC-4D8B-AFD0-D98EB20575C3}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{0468C0FD-CD61-4D45-8CEE-7AD439EC0420}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3507,15 +4655,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
@@ -3524,6 +4663,15 @@
     <TaxCatchAll xmlns="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3546,14 +4694,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A71CC56E-C3CE-4103-A70F-BE5CD4A5A2E6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3562,4 +4702,12 @@
     <ds:schemaRef ds:uri="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF4DEB3-F270-4480-B933-1B059C0B0529}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changed functions in BLS script to account for LAU. Changed the config file for BLS. Wrote a translation file for Health_4.
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/About Indicators.xlsx
+++ b/Indicator_Gen/config/About Indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08092D6D-55C1-4E3E-81D4-A2BA58E12352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFAD9B25-99F7-4B14-8459-F0A13820A854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="192">
   <si>
     <t>Indicator</t>
   </si>
@@ -732,6 +732,27 @@
   </si>
   <si>
     <t>Travel Mode by Race</t>
+  </si>
+  <si>
+    <t>Health_1</t>
+  </si>
+  <si>
+    <t>Access to Grocery Stores</t>
+  </si>
+  <si>
+    <t>Accessibility_3</t>
+  </si>
+  <si>
+    <t>Auto Ownership</t>
+  </si>
+  <si>
+    <t>MOE Threshold</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Not sure if I can pull SE's yet</t>
   </si>
 </sst>
 </file>
@@ -1233,411 +1254,584 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E88C108-3781-4F95-A6AF-A4204BCDFF66}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C1" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="C8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="C9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="C10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="C11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="C13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="C15" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="C16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="C17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="C18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="C19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="C20" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="C21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="C22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="C23" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="C24" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="C25" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="C26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="C27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="C28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="C29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="C30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>58</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="C31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>59</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="C32" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="C33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>63</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="C34" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>65</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="C35" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>67</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="C36" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>69</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="C37" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>71</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="C38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>73</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="C39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>75</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="C40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>77</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="C41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>79</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="C42" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>81</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="C43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>83</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="C44">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>85</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="C45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>87</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="C46" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>89</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="C47" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>139</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+      <c r="C48">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>183</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="C49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+      <c r="C50">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>187</v>
+      </c>
+      <c r="B51" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>181</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B52" t="s">
         <v>182</v>
+      </c>
+      <c r="C52">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>